<commit_message>
Woodwork pricing: item 1 TV unit with sliding door and fireplace, 500x300 cm
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XetM4kyjR9aszSEJL8QQpn
</commit_message>
<xml_diff>
--- a/assets/docs/woodwork-pricing.xlsx
+++ b/assets/docs/woodwork-pricing.xlsx
@@ -83,7 +83,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -105,11 +105,55 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -150,6 +194,8 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -534,6 +580,13 @@
           <t>مقدمة وملخص تصنيفات أعمال المشروع</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="15" t="n"/>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -541,6 +594,13 @@
           <t>تم تقسيم أعمال النجارة إلى بندين رئيسيين: أعمال النجارة (وحدات العرض ولايت بوكس ووحدات الخدمة)، والسقف المشدود (خشب ويشمل الوايرات والتعليق). يتم إدخال الكمية وسعر الوحدة لكل بند ويُحسب الإجمالي تلقائياً.</t>
         </is>
       </c>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="n"/>
+      <c r="F2" s="14" t="n"/>
+      <c r="G2" s="14" t="n"/>
+      <c r="H2" s="15" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -553,10 +613,10 @@
           <t>البند</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n"/>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="15" t="n"/>
       <c r="G3" s="1" t="inlineStr">
         <is>
           <t>الإجمالي</t>
@@ -577,10 +637,10 @@
           <t>أعمال النجارة</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
+      <c r="F4" s="15" t="n"/>
       <c r="G4" s="4">
         <f>'اعمال النجارة'!G19</f>
         <v/>
@@ -596,10 +656,10 @@
           <t>السقف المشدود (خشب و يشمل الوايرات و التعليق)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+      <c r="C5" s="14" t="n"/>
+      <c r="D5" s="14" t="n"/>
+      <c r="E5" s="14" t="n"/>
+      <c r="F5" s="15" t="n"/>
       <c r="G5" s="4">
         <f>'اعمال النجارة'!G25</f>
         <v/>
@@ -613,10 +673,10 @@
           <t>الإجمالي العام</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="15" t="n"/>
       <c r="G6" s="6">
         <f>G4+G5</f>
         <v/>
@@ -716,23 +776,26 @@
       <c r="G2" s="7" t="n"/>
       <c r="H2" s="7" t="n"/>
     </row>
-    <row r="3" ht="95" customHeight="1">
+    <row r="3" ht="110" customHeight="1">
       <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>وحدات العرض</t>
+          <t>وحدة تلفزيون</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>توريد وتركيب وحدة عرض [الكود]:
-[وصف الخامة والتشطيب والأبعاد حسب المخططات المعتمدة]
+          <t>توريد وتركيب وحدة مكتب التلفزيون مع باب سحاب ومكان للمدفأة:
+وحدة خشبية لمنطقة التلفزيون بمقاس 500×300 سم (العرض × الارتفاع) بدون المدفأة، مع باب سحاب، وتجهيز فتحة المدفأة حسب المخططات المعتمدة.
+لا يشمل البند توريد المدفأة.
 يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
         </is>
       </c>
-      <c r="D3" s="9" t="n"/>
+      <c r="D3" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>عدد</t>

</xml_diff>

<commit_message>
Woodwork pricing: items 2-4 (movable partition, bookcase with hidden door, majlis sliding door)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XetM4kyjR9aszSEJL8QQpn
</commit_message>
<xml_diff>
--- a/assets/docs/woodwork-pricing.xlsx
+++ b/assets/docs/woodwork-pricing.xlsx
@@ -808,23 +808,25 @@
       </c>
       <c r="H3" s="3" t="n"/>
     </row>
-    <row r="4" ht="95" customHeight="1">
+    <row r="4" ht="110" customHeight="1">
       <c r="A4" s="3" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>وحدات العرض</t>
+          <t>بارتيشن</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>توريد وتركيب وحدة عرض [الكود]:
-[وصف الخامة والتشطيب والأبعاد حسب المخططات المعتمدة]
+          <t>توريد وتركيب بارتيشن متحرك:
+بارتيشن متحرك بمقاس 240 سم × 300 سم (العرض × الارتفاع) حسب المخططات المعتمدة.
 يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n"/>
+      <c r="D4" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -837,23 +839,25 @@
       </c>
       <c r="H4" s="3" t="n"/>
     </row>
-    <row r="5" ht="95" customHeight="1">
+    <row r="5" ht="110" customHeight="1">
       <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>وحدات العرض</t>
+          <t>مكتبة</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>توريد وتركيب وحدة عرض [الكود]:
-[وصف الخامة والتشطيب والأبعاد حسب المخططات المعتمدة]
+          <t>توريد وتركيب مكتبة رفوف مع باب مخفي:
+مكتبة رفوف بمقاس 400 سم × 300 سم (العرض × الارتفاع) مع باب مخفي مدمج في الرفوف حسب المخططات المعتمدة.
 يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n"/>
+      <c r="D5" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -866,23 +870,26 @@
       </c>
       <c r="H5" s="3" t="n"/>
     </row>
-    <row r="6" ht="95" customHeight="1">
+    <row r="6" ht="110" customHeight="1">
       <c r="A6" s="3" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>لايت بوكس</t>
+          <t>باب</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>توريد وتركيب لايت بوكس خشبي بأبعاد [العرض×الارتفاع] سم:
-[وصف]
-يشمل البند الأعمال الخشبية وتركيب الليد فقط دون توريده.</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n"/>
+          <t>توريد وتركيب باب سحاب لمجلس الرجال:
+باب سحاب بمقاس 165 سم × 300 سم (العرض × الارتفاع) حسب المخططات المعتمدة.
+لا يشمل البند التلبيس (بند مستقل).
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>عدد</t>

</xml_diff>

<commit_message>
Woodwork pricing: majlis item 4 split into sub-items 4.1-4.4
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XetM4kyjR9aszSEJL8QQpn
</commit_message>
<xml_diff>
--- a/assets/docs/woodwork-pricing.xlsx
+++ b/assets/docs/woodwork-pricing.xlsx
@@ -870,55 +870,47 @@
       </c>
       <c r="H5" s="3" t="n"/>
     </row>
-    <row r="6" ht="110" customHeight="1">
-      <c r="A6" s="3" t="n">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>مجلس الرجال</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>أعمال مجلس الرجال</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="95" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>باب</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>توريد وتركيب باب سحاب لمجلس الرجال:
 باب سحاب بمقاس 165 سم × 300 سم (العرض × الارتفاع) حسب المخططات المعتمدة.
-لا يشمل البند التلبيس (بند مستقل).
 يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>عدد</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="4">
-        <f>D6*F6</f>
-        <v/>
-      </c>
-      <c r="H6" s="3" t="n"/>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>لايت بوكس</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>توريد وتركيب لايت بوكس خشبي بأبعاد [العرض×الارتفاع] سم:
-[وصف]
-يشمل البند الأعمال الخشبية وتركيب الليد فقط دون توريده.</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="n"/>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -932,22 +924,26 @@
       <c r="H7" s="3" t="n"/>
     </row>
     <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="3" t="n">
-        <v>6</v>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>لايت بوكس</t>
+          <t>تلبيس</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>توريد وتركيب لايت بوكس خشبي بأبعاد [العرض×الارتفاع] سم:
-[وصف]
-يشمل البند الأعمال الخشبية وتركيب الليد فقط دون توريده.</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n"/>
+          <t>توريد وتركيب تلبيس للباب المخفي:
+تلبيس بمقاس 200 سم × 300 سم (العرض × الارتفاع) حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -961,79 +957,87 @@
       <c r="H8" s="3" t="n"/>
     </row>
     <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="3" t="n">
-        <v>7</v>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
+          <t>دولاب عبايات</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>توريد وتركيب دولاب عبايات:
+دولاب بمقاس 330 سم × 330 سم (العرض × الارتفاع) وعمق 90 سم حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>عدد</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="4">
+        <f>D9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="95" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>دولاب عبايات</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>توريد وتركيب دولاب عبايات (2):
+دولاب بمقاس 250 سم × 300 سم (العرض × الارتفاع) حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>عدد</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="4">
+        <f>D10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
           <t>وحدة خدمة</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>توريد وتركيب وحدة خدمة [الكود]:
 [وصف الخامة والتشطيب والأبعاد]
 يشمل البند جميع أعمال التوريد والتركيب والتثبيت.</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>عدد</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="4">
-        <f>D9*F9</f>
-        <v/>
-      </c>
-      <c r="H9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>وحدة خدمة</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>توريد وتركيب وحدة خدمة [الكود]:
-[وصف الخامة والتشطيب والأبعاد]
-يشمل البند جميع أعمال التوريد والتركيب والتثبيت.</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>عدد</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="4">
-        <f>D10*F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="3" t="n"/>
-    </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>وحدة خدمة</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>توريد وتركيب وحدة خدمة [الكود]:
-[وصف الخامة والتشطيب والأبعاد]
-يشمل البند جميع أعمال التوريد والتركيب والتثبيت.</t>
-        </is>
-      </c>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -1049,7 +1053,7 @@
     </row>
     <row r="12" ht="95" customHeight="1">
       <c r="A12" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1077,7 +1081,7 @@
     </row>
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B13" s="3" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr"/>
@@ -1096,7 +1100,7 @@
     </row>
     <row r="14" ht="95" customHeight="1">
       <c r="A14" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr"/>
@@ -1115,7 +1119,7 @@
     </row>
     <row r="15" ht="95" customHeight="1">
       <c r="A15" s="3" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr"/>
@@ -1134,7 +1138,7 @@
     </row>
     <row r="16" ht="95" customHeight="1">
       <c r="A16" s="3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B16" s="3" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr"/>
@@ -1153,7 +1157,7 @@
     </row>
     <row r="17" ht="95" customHeight="1">
       <c r="A17" s="3" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B17" s="3" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr"/>
@@ -1172,7 +1176,7 @@
     </row>
     <row r="18" ht="95" customHeight="1">
       <c r="A18" s="3" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B18" s="3" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Woodwork pricing: item 5 Ghaida room with sub-items 5.1-5.5
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XetM4kyjR9aszSEJL8QQpn
</commit_message>
<xml_diff>
--- a/assets/docs/woodwork-pricing.xlsx
+++ b/assets/docs/woodwork-pricing.xlsx
@@ -1022,54 +1022,50 @@
       </c>
       <c r="H10" s="3" t="n"/>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="3" t="n">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>وحدة خدمة</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>توريد وتركيب وحدة خدمة [الكود]:
-[وصف الخامة والتشطيب والأبعاد]
-يشمل البند جميع أعمال التوريد والتركيب والتثبيت.</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>عدد</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="4">
-        <f>D11*F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="3" t="n"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>غرفة غيداء</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>أعمال غرفة غيداء</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
     </row>
     <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="3" t="n">
-        <v>6</v>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>وحدة عرض</t>
+          <t>أرفف</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>توريد وتركيب وحدات جدارية [وصف]
-لا يشمل البند توريد الليد، ويشمل تركيبه فقط.</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n"/>
+          <t>توريد وتركيب أرفف بجوار الدولاب:
+أرفف خشبية بمقاس 45 سم × 270 سم حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>متر مربع</t>
+          <t>عدد</t>
         </is>
       </c>
       <c r="F12" s="10" t="n"/>
@@ -1080,12 +1076,26 @@
       <c r="H12" s="3" t="n"/>
     </row>
     <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="9" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>تخزين فوق الدولاب</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>توريد وتركيب تخزين فوق الدولاب:
+وحدة تخزين بمقاس 63 سم × 400 سم حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -1099,12 +1109,27 @@
       <c r="H13" s="3" t="n"/>
     </row>
     <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="9" t="n"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>علبة أرفف</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>توريد وتركيب علبة أرفف بدون إضاءة:
+علبة أرفف بمقاس 43.5 سم × 310 سم حسب المخططات المعتمدة.
+لا يشمل البند الإضاءة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -1118,12 +1143,26 @@
       <c r="H14" s="3" t="n"/>
     </row>
     <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="9" t="n"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>تخزين فوق الدولاب</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>توريد وتركيب تخزين فوق الدولاب:
+وحدة تخزين بمقاس 300 سم × 63 سم حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -1137,12 +1176,26 @@
       <c r="H15" s="3" t="n"/>
     </row>
     <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="9" t="n"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>تخزين فوق الدولاب</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>توريد وتركيب تخزين فوق الدولاب (2):
+وحدة تخزين بمقاس 200 سم × 360 سم وعمق 36 سم حسب المخططات المعتمدة.
+يشمل البند جميع أعمال التوريد والتركيب والتثبيت اللازمة لإتمام العمل وفق التصميم المعتمد.</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
           <t>عدد</t>
@@ -1157,10 +1210,10 @@
     </row>
     <row r="17" ht="95" customHeight="1">
       <c r="A17" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="2" t="n"/>
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="3" t="inlineStr">
         <is>
@@ -1176,10 +1229,10 @@
     </row>
     <row r="18" ht="95" customHeight="1">
       <c r="A18" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="2" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="3" t="inlineStr">
         <is>

</xml_diff>